<commit_message>
Not yet half-ready implementations of a new 2D log curve data model, and more "new" data models
</commit_message>
<xml_diff>
--- a/excels/project_table.xlsx
+++ b/excels/project_table.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eribli\PycharmProjects\blixt_rp\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marte\PycharmProjects\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E6CD3A0-082E-4DF9-A490-1C0854E1BABA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8140177-F1DA-4ADB-896F-F3F812C0CD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14175" yWindow="4755" windowWidth="23535" windowHeight="13200" tabRatio="685" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2130" yWindow="14415" windowWidth="34695" windowHeight="12525" tabRatio="685" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
     <sheet name="Well logs" sheetId="2" r:id="rId2"/>
     <sheet name="Well paths" sheetId="3" r:id="rId3"/>
-    <sheet name="Checkshots" sheetId="4" r:id="rId4"/>
-    <sheet name="Regressions" sheetId="5" r:id="rId5"/>
-    <sheet name="Working intervals" sheetId="6" r:id="rId6"/>
-    <sheet name="Templates" sheetId="7" r:id="rId7"/>
+    <sheet name="Templates" sheetId="7" r:id="rId4"/>
+    <sheet name="Checkshots" sheetId="4" r:id="rId5"/>
+    <sheet name="Regressions" sheetId="5" r:id="rId6"/>
+    <sheet name="Working intervals" sheetId="6" r:id="rId7"/>
     <sheet name="Fluids" sheetId="8" r:id="rId8"/>
     <sheet name="Fluid mixtures" sheetId="9" r:id="rId9"/>
     <sheet name="Minerals" sheetId="10" r:id="rId10"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="912" uniqueCount="392">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="913" uniqueCount="393">
   <si>
     <t>Select Yes or No</t>
   </si>
@@ -1250,6 +1250,9 @@
   </si>
   <si>
     <t>Observation or model (name)</t>
+  </si>
+  <si>
+    <t>marker</t>
   </si>
 </sst>
 </file>
@@ -4039,6 +4042,981 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
+  <dimension ref="A1:O30"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="14.140625" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="I2" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="J2" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="K2" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="M2" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="N2" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="O2" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B3" t="s">
+        <v>55</v>
+      </c>
+      <c r="C3" t="s">
+        <v>203</v>
+      </c>
+      <c r="D3" t="s">
+        <v>204</v>
+      </c>
+      <c r="E3" t="s">
+        <v>205</v>
+      </c>
+      <c r="F3" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="G3" s="3">
+        <v>200</v>
+      </c>
+      <c r="I3" t="s">
+        <v>206</v>
+      </c>
+      <c r="K3" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="L3" t="s">
+        <v>207</v>
+      </c>
+      <c r="M3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E4" t="s">
+        <v>205</v>
+      </c>
+      <c r="F4" s="3">
+        <v>3500</v>
+      </c>
+      <c r="G4" s="3">
+        <v>4800</v>
+      </c>
+      <c r="I4" t="s">
+        <v>206</v>
+      </c>
+      <c r="K4" s="15" t="s">
+        <v>16</v>
+      </c>
+      <c r="L4" t="s">
+        <v>207</v>
+      </c>
+      <c r="M4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C5" t="s">
+        <v>208</v>
+      </c>
+      <c r="D5" t="s">
+        <v>209</v>
+      </c>
+      <c r="E5" t="s">
+        <v>205</v>
+      </c>
+      <c r="F5" s="3">
+        <v>1800</v>
+      </c>
+      <c r="G5" s="3">
+        <v>3000</v>
+      </c>
+      <c r="I5" t="s">
+        <v>206</v>
+      </c>
+      <c r="K5" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="L5" t="s">
+        <v>207</v>
+      </c>
+      <c r="M5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>210</v>
+      </c>
+      <c r="B6" t="s">
+        <v>211</v>
+      </c>
+      <c r="C6" t="s">
+        <v>212</v>
+      </c>
+      <c r="D6" t="s">
+        <v>204</v>
+      </c>
+      <c r="E6" t="s">
+        <v>205</v>
+      </c>
+      <c r="F6" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="G6" s="3">
+        <v>2000</v>
+      </c>
+      <c r="I6" t="s">
+        <v>206</v>
+      </c>
+      <c r="K6" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="L6" t="s">
+        <v>207</v>
+      </c>
+      <c r="M6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>213</v>
+      </c>
+      <c r="B7" t="s">
+        <v>214</v>
+      </c>
+      <c r="C7" t="s">
+        <v>207</v>
+      </c>
+      <c r="D7" t="s">
+        <v>209</v>
+      </c>
+      <c r="E7" t="s">
+        <v>205</v>
+      </c>
+      <c r="F7" s="3">
+        <v>1.4</v>
+      </c>
+      <c r="G7" s="3">
+        <v>4</v>
+      </c>
+      <c r="I7" t="s">
+        <v>206</v>
+      </c>
+      <c r="K7" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="L7" t="s">
+        <v>207</v>
+      </c>
+      <c r="M7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>215</v>
+      </c>
+      <c r="B8" t="s">
+        <v>216</v>
+      </c>
+      <c r="C8" t="s">
+        <v>217</v>
+      </c>
+      <c r="D8" t="s">
+        <v>209</v>
+      </c>
+      <c r="E8" t="s">
+        <v>205</v>
+      </c>
+      <c r="F8" s="3">
+        <v>6500</v>
+      </c>
+      <c r="G8" s="3">
+        <v>11000</v>
+      </c>
+      <c r="I8" t="s">
+        <v>206</v>
+      </c>
+      <c r="K8" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="L8" t="s">
+        <v>207</v>
+      </c>
+      <c r="M8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>219</v>
+      </c>
+      <c r="C9" t="s">
+        <v>220</v>
+      </c>
+      <c r="D9" t="s">
+        <v>209</v>
+      </c>
+      <c r="E9" t="s">
+        <v>205</v>
+      </c>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="I9" t="s">
+        <v>206</v>
+      </c>
+      <c r="K9" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="M9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>221</v>
+      </c>
+      <c r="C10" t="s">
+        <v>220</v>
+      </c>
+      <c r="D10" t="s">
+        <v>209</v>
+      </c>
+      <c r="E10" t="s">
+        <v>205</v>
+      </c>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="I10" t="s">
+        <v>206</v>
+      </c>
+      <c r="K10" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="M10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>222</v>
+      </c>
+      <c r="B11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" t="s">
+        <v>207</v>
+      </c>
+      <c r="D11" t="s">
+        <v>209</v>
+      </c>
+      <c r="E11" t="s">
+        <v>205</v>
+      </c>
+      <c r="F11" s="3">
+        <v>0</v>
+      </c>
+      <c r="G11" s="3">
+        <v>0.3</v>
+      </c>
+      <c r="I11" t="s">
+        <v>206</v>
+      </c>
+      <c r="K11" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="L11" t="s">
+        <v>207</v>
+      </c>
+      <c r="M11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>223</v>
+      </c>
+      <c r="B12" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" t="s">
+        <v>207</v>
+      </c>
+      <c r="D12" t="s">
+        <v>209</v>
+      </c>
+      <c r="E12" t="s">
+        <v>205</v>
+      </c>
+      <c r="F12" s="3">
+        <v>0</v>
+      </c>
+      <c r="G12" s="3">
+        <v>1</v>
+      </c>
+      <c r="I12" t="s">
+        <v>206</v>
+      </c>
+      <c r="K12" s="26" t="s">
+        <v>224</v>
+      </c>
+      <c r="L12" t="s">
+        <v>225</v>
+      </c>
+      <c r="M12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>226</v>
+      </c>
+      <c r="B13" t="s">
+        <v>54</v>
+      </c>
+      <c r="C13" t="s">
+        <v>207</v>
+      </c>
+      <c r="D13" t="s">
+        <v>209</v>
+      </c>
+      <c r="E13" t="s">
+        <v>205</v>
+      </c>
+      <c r="F13" s="3">
+        <v>0</v>
+      </c>
+      <c r="G13" s="3">
+        <v>1</v>
+      </c>
+      <c r="I13" t="s">
+        <v>206</v>
+      </c>
+      <c r="K13" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="L13" t="s">
+        <v>207</v>
+      </c>
+      <c r="M13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>77</v>
+      </c>
+      <c r="B14" t="s">
+        <v>50</v>
+      </c>
+      <c r="C14" t="s">
+        <v>227</v>
+      </c>
+      <c r="D14" t="s">
+        <v>209</v>
+      </c>
+      <c r="E14" t="s">
+        <v>205</v>
+      </c>
+      <c r="F14" s="3">
+        <v>2</v>
+      </c>
+      <c r="G14" s="3">
+        <v>3</v>
+      </c>
+      <c r="I14" t="s">
+        <v>206</v>
+      </c>
+      <c r="K14" s="23" t="s">
+        <v>39</v>
+      </c>
+      <c r="L14" t="s">
+        <v>207</v>
+      </c>
+      <c r="M14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>228</v>
+      </c>
+      <c r="B15" t="s">
+        <v>51</v>
+      </c>
+      <c r="C15" t="s">
+        <v>229</v>
+      </c>
+      <c r="D15" t="s">
+        <v>209</v>
+      </c>
+      <c r="E15" t="s">
+        <v>205</v>
+      </c>
+      <c r="F15" s="3">
+        <v>0.45</v>
+      </c>
+      <c r="G15" s="3">
+        <v>-0.15</v>
+      </c>
+      <c r="I15" t="s">
+        <v>206</v>
+      </c>
+      <c r="K15" s="27" t="s">
+        <v>230</v>
+      </c>
+      <c r="L15" t="s">
+        <v>207</v>
+      </c>
+      <c r="M15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>231</v>
+      </c>
+      <c r="B16" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" t="s">
+        <v>232</v>
+      </c>
+      <c r="D16" t="s">
+        <v>209</v>
+      </c>
+      <c r="E16" t="s">
+        <v>205</v>
+      </c>
+      <c r="F16" s="3">
+        <v>6</v>
+      </c>
+      <c r="G16" s="3">
+        <v>10</v>
+      </c>
+      <c r="I16" t="s">
+        <v>206</v>
+      </c>
+      <c r="K16" s="24" t="s">
+        <v>233</v>
+      </c>
+      <c r="L16" t="s">
+        <v>207</v>
+      </c>
+      <c r="M16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>234</v>
+      </c>
+      <c r="B17" t="s">
+        <v>49</v>
+      </c>
+      <c r="C17" t="s">
+        <v>235</v>
+      </c>
+      <c r="D17" t="s">
+        <v>209</v>
+      </c>
+      <c r="E17" t="s">
+        <v>205</v>
+      </c>
+      <c r="F17" s="3">
+        <v>0</v>
+      </c>
+      <c r="G17" s="3">
+        <v>350</v>
+      </c>
+      <c r="I17" t="s">
+        <v>206</v>
+      </c>
+      <c r="K17" s="25" t="s">
+        <v>236</v>
+      </c>
+      <c r="L17" t="s">
+        <v>207</v>
+      </c>
+      <c r="M17">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>237</v>
+      </c>
+      <c r="B18" t="s">
+        <v>46</v>
+      </c>
+      <c r="C18" t="s">
+        <v>238</v>
+      </c>
+      <c r="D18" t="s">
+        <v>209</v>
+      </c>
+      <c r="E18" t="s">
+        <v>205</v>
+      </c>
+      <c r="F18" s="3">
+        <v>40</v>
+      </c>
+      <c r="G18" s="3">
+        <v>150</v>
+      </c>
+      <c r="I18" t="s">
+        <v>206</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>19</v>
+      </c>
+      <c r="L18" t="s">
+        <v>207</v>
+      </c>
+      <c r="M18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>239</v>
+      </c>
+      <c r="B19" t="s">
+        <v>240</v>
+      </c>
+      <c r="C19" t="s">
+        <v>238</v>
+      </c>
+      <c r="D19" t="s">
+        <v>209</v>
+      </c>
+      <c r="E19" t="s">
+        <v>205</v>
+      </c>
+      <c r="F19" s="3">
+        <v>80</v>
+      </c>
+      <c r="G19" s="3">
+        <v>300</v>
+      </c>
+      <c r="I19" t="s">
+        <v>206</v>
+      </c>
+      <c r="K19" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="L19" t="s">
+        <v>207</v>
+      </c>
+      <c r="M19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>241</v>
+      </c>
+      <c r="B20" t="s">
+        <v>241</v>
+      </c>
+      <c r="C20" t="s">
+        <v>242</v>
+      </c>
+      <c r="D20" t="s">
+        <v>209</v>
+      </c>
+      <c r="E20" t="s">
+        <v>205</v>
+      </c>
+      <c r="F20" s="3">
+        <v>0</v>
+      </c>
+      <c r="G20" s="3">
+        <v>15</v>
+      </c>
+      <c r="I20" t="s">
+        <v>206</v>
+      </c>
+      <c r="K20" s="18" t="s">
+        <v>29</v>
+      </c>
+      <c r="L20" t="s">
+        <v>207</v>
+      </c>
+      <c r="M20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>243</v>
+      </c>
+      <c r="B21" t="s">
+        <v>244</v>
+      </c>
+      <c r="C21" t="s">
+        <v>242</v>
+      </c>
+      <c r="D21" t="s">
+        <v>245</v>
+      </c>
+      <c r="E21" t="s">
+        <v>205</v>
+      </c>
+      <c r="F21" s="3">
+        <v>0</v>
+      </c>
+      <c r="G21" s="3">
+        <v>5</v>
+      </c>
+      <c r="I21" t="s">
+        <v>246</v>
+      </c>
+      <c r="J21" t="s">
+        <v>247</v>
+      </c>
+      <c r="K21" s="19" t="s">
+        <v>218</v>
+      </c>
+      <c r="L21" t="s">
+        <v>207</v>
+      </c>
+      <c r="M21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>248</v>
+      </c>
+      <c r="B22" t="s">
+        <v>249</v>
+      </c>
+      <c r="C22" t="s">
+        <v>207</v>
+      </c>
+      <c r="D22" t="s">
+        <v>209</v>
+      </c>
+      <c r="F22" s="3">
+        <v>0</v>
+      </c>
+      <c r="G22" s="3">
+        <v>900</v>
+      </c>
+      <c r="K22" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="L22" t="s">
+        <v>207</v>
+      </c>
+      <c r="M22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>250</v>
+      </c>
+      <c r="B23" t="s">
+        <v>251</v>
+      </c>
+      <c r="C23" t="s">
+        <v>207</v>
+      </c>
+      <c r="D23" t="s">
+        <v>245</v>
+      </c>
+      <c r="F23" s="3">
+        <v>0</v>
+      </c>
+      <c r="G23" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="I23" t="s">
+        <v>252</v>
+      </c>
+      <c r="J23" t="s">
+        <v>253</v>
+      </c>
+      <c r="K23" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="L23" t="s">
+        <v>207</v>
+      </c>
+      <c r="M23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>254</v>
+      </c>
+      <c r="B24" t="s">
+        <v>255</v>
+      </c>
+      <c r="C24" t="s">
+        <v>256</v>
+      </c>
+      <c r="D24" t="s">
+        <v>209</v>
+      </c>
+      <c r="E24" t="s">
+        <v>205</v>
+      </c>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="I24" t="s">
+        <v>206</v>
+      </c>
+      <c r="K24" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="L24" t="s">
+        <v>225</v>
+      </c>
+      <c r="M24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>257</v>
+      </c>
+      <c r="B25" t="s">
+        <v>258</v>
+      </c>
+      <c r="C25" t="s">
+        <v>232</v>
+      </c>
+      <c r="D25" t="s">
+        <v>209</v>
+      </c>
+      <c r="E25" t="s">
+        <v>205</v>
+      </c>
+      <c r="F25" s="3">
+        <v>4</v>
+      </c>
+      <c r="G25" s="3">
+        <v>12</v>
+      </c>
+      <c r="I25" t="s">
+        <v>206</v>
+      </c>
+      <c r="K25" s="24" t="s">
+        <v>233</v>
+      </c>
+      <c r="L25" t="s">
+        <v>225</v>
+      </c>
+      <c r="M25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B26" t="s">
+        <v>57</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1</v>
+      </c>
+      <c r="D26" t="s">
+        <v>209</v>
+      </c>
+      <c r="E26" t="s">
+        <v>205</v>
+      </c>
+      <c r="I26" t="s">
+        <v>206</v>
+      </c>
+      <c r="K26" s="24" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B27" t="s">
+        <v>259</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1</v>
+      </c>
+      <c r="D27" t="s">
+        <v>209</v>
+      </c>
+      <c r="E27" t="s">
+        <v>205</v>
+      </c>
+      <c r="I27" t="s">
+        <v>206</v>
+      </c>
+      <c r="K27" s="24" t="s">
+        <v>233</v>
+      </c>
+      <c r="L27" t="s">
+        <v>207</v>
+      </c>
+      <c r="M27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>260</v>
+      </c>
+      <c r="B28" t="s">
+        <v>261</v>
+      </c>
+      <c r="C28" t="s">
+        <v>17</v>
+      </c>
+      <c r="D28" t="s">
+        <v>209</v>
+      </c>
+      <c r="E28" t="s">
+        <v>205</v>
+      </c>
+      <c r="I28" t="s">
+        <v>206</v>
+      </c>
+      <c r="K28" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="L28" t="s">
+        <v>207</v>
+      </c>
+      <c r="M28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>262</v>
+      </c>
+      <c r="B29" t="s">
+        <v>263</v>
+      </c>
+      <c r="C29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29" t="s">
+        <v>209</v>
+      </c>
+      <c r="E29" t="s">
+        <v>205</v>
+      </c>
+      <c r="I29" t="s">
+        <v>206</v>
+      </c>
+      <c r="K29" s="22" t="s">
+        <v>37</v>
+      </c>
+      <c r="L29" t="s">
+        <v>207</v>
+      </c>
+      <c r="M29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="B30" t="s">
+        <v>264</v>
+      </c>
+      <c r="C30" t="s">
+        <v>207</v>
+      </c>
+      <c r="D30" t="s">
+        <v>209</v>
+      </c>
+      <c r="E30" t="s">
+        <v>205</v>
+      </c>
+      <c r="I30" t="s">
+        <v>265</v>
+      </c>
+      <c r="K30" s="36" t="s">
+        <v>266</v>
+      </c>
+      <c r="L30" t="s">
+        <v>207</v>
+      </c>
+      <c r="M30">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations disablePrompts="1" count="1">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="L3:L30" xr:uid="{00000000-0002-0000-0600-000000000000}">
+      <formula1>LineStyles</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4263,7 +5241,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:M17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -4725,7 +5703,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5409,978 +6387,6 @@
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:N30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>197</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>199</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>200</v>
-      </c>
-      <c r="N2" s="1" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>202</v>
-      </c>
-      <c r="B3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C3" t="s">
-        <v>203</v>
-      </c>
-      <c r="D3" t="s">
-        <v>204</v>
-      </c>
-      <c r="E3" t="s">
-        <v>205</v>
-      </c>
-      <c r="F3" s="3">
-        <v>0.2</v>
-      </c>
-      <c r="G3" s="3">
-        <v>200</v>
-      </c>
-      <c r="I3" t="s">
-        <v>206</v>
-      </c>
-      <c r="K3" s="14" t="s">
-        <v>13</v>
-      </c>
-      <c r="L3" t="s">
-        <v>207</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B4" t="s">
-        <v>45</v>
-      </c>
-      <c r="C4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D4" t="s">
-        <v>209</v>
-      </c>
-      <c r="E4" t="s">
-        <v>205</v>
-      </c>
-      <c r="F4" s="3">
-        <v>3500</v>
-      </c>
-      <c r="G4" s="3">
-        <v>4800</v>
-      </c>
-      <c r="I4" t="s">
-        <v>206</v>
-      </c>
-      <c r="K4" s="15" t="s">
-        <v>16</v>
-      </c>
-      <c r="L4" t="s">
-        <v>207</v>
-      </c>
-      <c r="M4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B5" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" t="s">
-        <v>208</v>
-      </c>
-      <c r="D5" t="s">
-        <v>209</v>
-      </c>
-      <c r="E5" t="s">
-        <v>205</v>
-      </c>
-      <c r="F5" s="3">
-        <v>1800</v>
-      </c>
-      <c r="G5" s="3">
-        <v>3000</v>
-      </c>
-      <c r="I5" t="s">
-        <v>206</v>
-      </c>
-      <c r="K5" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="L5" t="s">
-        <v>207</v>
-      </c>
-      <c r="M5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>210</v>
-      </c>
-      <c r="B6" t="s">
-        <v>211</v>
-      </c>
-      <c r="C6" t="s">
-        <v>212</v>
-      </c>
-      <c r="D6" t="s">
-        <v>204</v>
-      </c>
-      <c r="E6" t="s">
-        <v>205</v>
-      </c>
-      <c r="F6" s="3">
-        <v>0.01</v>
-      </c>
-      <c r="G6" s="3">
-        <v>2000</v>
-      </c>
-      <c r="I6" t="s">
-        <v>206</v>
-      </c>
-      <c r="K6" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="L6" t="s">
-        <v>207</v>
-      </c>
-      <c r="M6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>213</v>
-      </c>
-      <c r="B7" t="s">
-        <v>214</v>
-      </c>
-      <c r="C7" t="s">
-        <v>207</v>
-      </c>
-      <c r="D7" t="s">
-        <v>209</v>
-      </c>
-      <c r="E7" t="s">
-        <v>205</v>
-      </c>
-      <c r="F7" s="3">
-        <v>1.4</v>
-      </c>
-      <c r="G7" s="3">
-        <v>4</v>
-      </c>
-      <c r="I7" t="s">
-        <v>206</v>
-      </c>
-      <c r="K7" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="L7" t="s">
-        <v>207</v>
-      </c>
-      <c r="M7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>215</v>
-      </c>
-      <c r="B8" t="s">
-        <v>216</v>
-      </c>
-      <c r="C8" t="s">
-        <v>217</v>
-      </c>
-      <c r="D8" t="s">
-        <v>209</v>
-      </c>
-      <c r="E8" t="s">
-        <v>205</v>
-      </c>
-      <c r="F8" s="3">
-        <v>6500</v>
-      </c>
-      <c r="G8" s="3">
-        <v>11000</v>
-      </c>
-      <c r="I8" t="s">
-        <v>206</v>
-      </c>
-      <c r="K8" s="19" t="s">
-        <v>218</v>
-      </c>
-      <c r="L8" t="s">
-        <v>207</v>
-      </c>
-      <c r="M8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B9" t="s">
-        <v>219</v>
-      </c>
-      <c r="C9" t="s">
-        <v>220</v>
-      </c>
-      <c r="D9" t="s">
-        <v>209</v>
-      </c>
-      <c r="E9" t="s">
-        <v>205</v>
-      </c>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
-      <c r="I9" t="s">
-        <v>206</v>
-      </c>
-      <c r="K9" s="19" t="s">
-        <v>218</v>
-      </c>
-      <c r="M9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B10" t="s">
-        <v>221</v>
-      </c>
-      <c r="C10" t="s">
-        <v>220</v>
-      </c>
-      <c r="D10" t="s">
-        <v>209</v>
-      </c>
-      <c r="E10" t="s">
-        <v>205</v>
-      </c>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="I10" t="s">
-        <v>206</v>
-      </c>
-      <c r="K10" s="19" t="s">
-        <v>218</v>
-      </c>
-      <c r="M10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>222</v>
-      </c>
-      <c r="B11" t="s">
-        <v>52</v>
-      </c>
-      <c r="C11" t="s">
-        <v>207</v>
-      </c>
-      <c r="D11" t="s">
-        <v>209</v>
-      </c>
-      <c r="E11" t="s">
-        <v>205</v>
-      </c>
-      <c r="F11" s="3">
-        <v>0</v>
-      </c>
-      <c r="G11" s="3">
-        <v>0.3</v>
-      </c>
-      <c r="I11" t="s">
-        <v>206</v>
-      </c>
-      <c r="K11" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="L11" t="s">
-        <v>207</v>
-      </c>
-      <c r="M11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>223</v>
-      </c>
-      <c r="B12" t="s">
-        <v>53</v>
-      </c>
-      <c r="C12" t="s">
-        <v>207</v>
-      </c>
-      <c r="D12" t="s">
-        <v>209</v>
-      </c>
-      <c r="E12" t="s">
-        <v>205</v>
-      </c>
-      <c r="F12" s="3">
-        <v>0</v>
-      </c>
-      <c r="G12" s="3">
-        <v>1</v>
-      </c>
-      <c r="I12" t="s">
-        <v>206</v>
-      </c>
-      <c r="K12" s="26" t="s">
-        <v>224</v>
-      </c>
-      <c r="L12" t="s">
-        <v>225</v>
-      </c>
-      <c r="M12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>226</v>
-      </c>
-      <c r="B13" t="s">
-        <v>54</v>
-      </c>
-      <c r="C13" t="s">
-        <v>207</v>
-      </c>
-      <c r="D13" t="s">
-        <v>209</v>
-      </c>
-      <c r="E13" t="s">
-        <v>205</v>
-      </c>
-      <c r="F13" s="3">
-        <v>0</v>
-      </c>
-      <c r="G13" s="3">
-        <v>1</v>
-      </c>
-      <c r="I13" t="s">
-        <v>206</v>
-      </c>
-      <c r="K13" s="22" t="s">
-        <v>37</v>
-      </c>
-      <c r="L13" t="s">
-        <v>207</v>
-      </c>
-      <c r="M13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>77</v>
-      </c>
-      <c r="B14" t="s">
-        <v>50</v>
-      </c>
-      <c r="C14" t="s">
-        <v>227</v>
-      </c>
-      <c r="D14" t="s">
-        <v>209</v>
-      </c>
-      <c r="E14" t="s">
-        <v>205</v>
-      </c>
-      <c r="F14" s="3">
-        <v>2</v>
-      </c>
-      <c r="G14" s="3">
-        <v>3</v>
-      </c>
-      <c r="I14" t="s">
-        <v>206</v>
-      </c>
-      <c r="K14" s="23" t="s">
-        <v>39</v>
-      </c>
-      <c r="L14" t="s">
-        <v>207</v>
-      </c>
-      <c r="M14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>228</v>
-      </c>
-      <c r="B15" t="s">
-        <v>51</v>
-      </c>
-      <c r="C15" t="s">
-        <v>229</v>
-      </c>
-      <c r="D15" t="s">
-        <v>209</v>
-      </c>
-      <c r="E15" t="s">
-        <v>205</v>
-      </c>
-      <c r="F15" s="3">
-        <v>0.45</v>
-      </c>
-      <c r="G15" s="3">
-        <v>-0.15</v>
-      </c>
-      <c r="I15" t="s">
-        <v>206</v>
-      </c>
-      <c r="K15" s="27" t="s">
-        <v>230</v>
-      </c>
-      <c r="L15" t="s">
-        <v>207</v>
-      </c>
-      <c r="M15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>231</v>
-      </c>
-      <c r="B16" t="s">
-        <v>56</v>
-      </c>
-      <c r="C16" t="s">
-        <v>232</v>
-      </c>
-      <c r="D16" t="s">
-        <v>209</v>
-      </c>
-      <c r="E16" t="s">
-        <v>205</v>
-      </c>
-      <c r="F16" s="3">
-        <v>6</v>
-      </c>
-      <c r="G16" s="3">
-        <v>10</v>
-      </c>
-      <c r="I16" t="s">
-        <v>206</v>
-      </c>
-      <c r="K16" s="24" t="s">
-        <v>233</v>
-      </c>
-      <c r="L16" t="s">
-        <v>207</v>
-      </c>
-      <c r="M16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>234</v>
-      </c>
-      <c r="B17" t="s">
-        <v>49</v>
-      </c>
-      <c r="C17" t="s">
-        <v>235</v>
-      </c>
-      <c r="D17" t="s">
-        <v>209</v>
-      </c>
-      <c r="E17" t="s">
-        <v>205</v>
-      </c>
-      <c r="F17" s="3">
-        <v>0</v>
-      </c>
-      <c r="G17" s="3">
-        <v>350</v>
-      </c>
-      <c r="I17" t="s">
-        <v>206</v>
-      </c>
-      <c r="K17" s="25" t="s">
-        <v>236</v>
-      </c>
-      <c r="L17" t="s">
-        <v>207</v>
-      </c>
-      <c r="M17">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>237</v>
-      </c>
-      <c r="B18" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18" t="s">
-        <v>238</v>
-      </c>
-      <c r="D18" t="s">
-        <v>209</v>
-      </c>
-      <c r="E18" t="s">
-        <v>205</v>
-      </c>
-      <c r="F18" s="3">
-        <v>40</v>
-      </c>
-      <c r="G18" s="3">
-        <v>150</v>
-      </c>
-      <c r="I18" t="s">
-        <v>206</v>
-      </c>
-      <c r="K18" s="16" t="s">
-        <v>19</v>
-      </c>
-      <c r="L18" t="s">
-        <v>207</v>
-      </c>
-      <c r="M18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>239</v>
-      </c>
-      <c r="B19" t="s">
-        <v>240</v>
-      </c>
-      <c r="C19" t="s">
-        <v>238</v>
-      </c>
-      <c r="D19" t="s">
-        <v>209</v>
-      </c>
-      <c r="E19" t="s">
-        <v>205</v>
-      </c>
-      <c r="F19" s="3">
-        <v>80</v>
-      </c>
-      <c r="G19" s="3">
-        <v>300</v>
-      </c>
-      <c r="I19" t="s">
-        <v>206</v>
-      </c>
-      <c r="K19" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="L19" t="s">
-        <v>207</v>
-      </c>
-      <c r="M19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>241</v>
-      </c>
-      <c r="B20" t="s">
-        <v>241</v>
-      </c>
-      <c r="C20" t="s">
-        <v>242</v>
-      </c>
-      <c r="D20" t="s">
-        <v>209</v>
-      </c>
-      <c r="E20" t="s">
-        <v>205</v>
-      </c>
-      <c r="F20" s="3">
-        <v>0</v>
-      </c>
-      <c r="G20" s="3">
-        <v>15</v>
-      </c>
-      <c r="I20" t="s">
-        <v>206</v>
-      </c>
-      <c r="K20" s="18" t="s">
-        <v>29</v>
-      </c>
-      <c r="L20" t="s">
-        <v>207</v>
-      </c>
-      <c r="M20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>243</v>
-      </c>
-      <c r="B21" t="s">
-        <v>244</v>
-      </c>
-      <c r="C21" t="s">
-        <v>242</v>
-      </c>
-      <c r="D21" t="s">
-        <v>245</v>
-      </c>
-      <c r="E21" t="s">
-        <v>205</v>
-      </c>
-      <c r="F21" s="3">
-        <v>0</v>
-      </c>
-      <c r="G21" s="3">
-        <v>5</v>
-      </c>
-      <c r="I21" t="s">
-        <v>246</v>
-      </c>
-      <c r="J21" t="s">
-        <v>247</v>
-      </c>
-      <c r="K21" s="19" t="s">
-        <v>218</v>
-      </c>
-      <c r="L21" t="s">
-        <v>207</v>
-      </c>
-      <c r="M21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>248</v>
-      </c>
-      <c r="B22" t="s">
-        <v>249</v>
-      </c>
-      <c r="C22" t="s">
-        <v>207</v>
-      </c>
-      <c r="D22" t="s">
-        <v>209</v>
-      </c>
-      <c r="F22" s="3">
-        <v>0</v>
-      </c>
-      <c r="G22" s="3">
-        <v>900</v>
-      </c>
-      <c r="K22" s="20" t="s">
-        <v>23</v>
-      </c>
-      <c r="L22" t="s">
-        <v>207</v>
-      </c>
-      <c r="M22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>250</v>
-      </c>
-      <c r="B23" t="s">
-        <v>251</v>
-      </c>
-      <c r="C23" t="s">
-        <v>207</v>
-      </c>
-      <c r="D23" t="s">
-        <v>245</v>
-      </c>
-      <c r="F23" s="3">
-        <v>0</v>
-      </c>
-      <c r="G23" s="3">
-        <v>0.5</v>
-      </c>
-      <c r="I23" t="s">
-        <v>252</v>
-      </c>
-      <c r="J23" t="s">
-        <v>253</v>
-      </c>
-      <c r="K23" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="L23" t="s">
-        <v>207</v>
-      </c>
-      <c r="M23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>254</v>
-      </c>
-      <c r="B24" t="s">
-        <v>255</v>
-      </c>
-      <c r="C24" t="s">
-        <v>256</v>
-      </c>
-      <c r="D24" t="s">
-        <v>209</v>
-      </c>
-      <c r="E24" t="s">
-        <v>205</v>
-      </c>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="I24" t="s">
-        <v>206</v>
-      </c>
-      <c r="K24" s="22" t="s">
-        <v>37</v>
-      </c>
-      <c r="L24" t="s">
-        <v>225</v>
-      </c>
-      <c r="M24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>257</v>
-      </c>
-      <c r="B25" t="s">
-        <v>258</v>
-      </c>
-      <c r="C25" t="s">
-        <v>232</v>
-      </c>
-      <c r="D25" t="s">
-        <v>209</v>
-      </c>
-      <c r="E25" t="s">
-        <v>205</v>
-      </c>
-      <c r="F25" s="3">
-        <v>4</v>
-      </c>
-      <c r="G25" s="3">
-        <v>12</v>
-      </c>
-      <c r="I25" t="s">
-        <v>206</v>
-      </c>
-      <c r="K25" s="24" t="s">
-        <v>233</v>
-      </c>
-      <c r="L25" t="s">
-        <v>225</v>
-      </c>
-      <c r="M25">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B26" t="s">
-        <v>57</v>
-      </c>
-      <c r="C26" t="s">
-        <v>1</v>
-      </c>
-      <c r="D26" t="s">
-        <v>209</v>
-      </c>
-      <c r="E26" t="s">
-        <v>205</v>
-      </c>
-      <c r="I26" t="s">
-        <v>206</v>
-      </c>
-      <c r="K26" s="24" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B27" t="s">
-        <v>259</v>
-      </c>
-      <c r="C27" t="s">
-        <v>1</v>
-      </c>
-      <c r="D27" t="s">
-        <v>209</v>
-      </c>
-      <c r="E27" t="s">
-        <v>205</v>
-      </c>
-      <c r="I27" t="s">
-        <v>206</v>
-      </c>
-      <c r="K27" s="24" t="s">
-        <v>233</v>
-      </c>
-      <c r="L27" t="s">
-        <v>207</v>
-      </c>
-      <c r="M27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>260</v>
-      </c>
-      <c r="B28" t="s">
-        <v>261</v>
-      </c>
-      <c r="C28" t="s">
-        <v>17</v>
-      </c>
-      <c r="D28" t="s">
-        <v>209</v>
-      </c>
-      <c r="E28" t="s">
-        <v>205</v>
-      </c>
-      <c r="I28" t="s">
-        <v>206</v>
-      </c>
-      <c r="K28" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="L28" t="s">
-        <v>207</v>
-      </c>
-      <c r="M28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>262</v>
-      </c>
-      <c r="B29" t="s">
-        <v>263</v>
-      </c>
-      <c r="C29" t="s">
-        <v>17</v>
-      </c>
-      <c r="D29" t="s">
-        <v>209</v>
-      </c>
-      <c r="E29" t="s">
-        <v>205</v>
-      </c>
-      <c r="I29" t="s">
-        <v>206</v>
-      </c>
-      <c r="K29" s="22" t="s">
-        <v>37</v>
-      </c>
-      <c r="L29" t="s">
-        <v>207</v>
-      </c>
-      <c r="M29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="B30" t="s">
-        <v>264</v>
-      </c>
-      <c r="C30" t="s">
-        <v>207</v>
-      </c>
-      <c r="D30" t="s">
-        <v>209</v>
-      </c>
-      <c r="E30" t="s">
-        <v>205</v>
-      </c>
-      <c r="I30" t="s">
-        <v>265</v>
-      </c>
-      <c r="K30" s="36" t="s">
-        <v>266</v>
-      </c>
-      <c r="L30" t="s">
-        <v>207</v>
-      </c>
-      <c r="M30">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations disablePrompts="1" count="1">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="L3:L30" xr:uid="{00000000-0002-0000-0600-000000000000}">
-      <formula1>LineStyles</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Loads of ongoing work
</commit_message>
<xml_diff>
--- a/excels/project_table.xlsx
+++ b/excels/project_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marte\PycharmProjects\blixt_rp\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emb\Documents\PycharmProjects\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F8140177-F1DA-4ADB-896F-F3F812C0CD3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5870F9E8-CBDA-4D8C-8DE7-5851E80CC5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2130" yWindow="14415" windowWidth="34695" windowHeight="12525" tabRatio="685" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30912" windowHeight="15588" tabRatio="685" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -6609,7 +6609,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
         <v>295</v>
@@ -6635,7 +6635,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
         <v>295</v>
@@ -6661,7 +6661,7 @@
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="31" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B6" s="31" t="s">
         <v>298</v>

</xml_diff>

<commit_message>
Mostly worked on PL1221.py
</commit_message>
<xml_diff>
--- a/excels/project_table.xlsx
+++ b/excels/project_table.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emb\Documents\PycharmProjects\blixt_rp\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5870F9E8-CBDA-4D8C-8DE7-5851E80CC5CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82A49DCD-8218-449B-8C5A-B03D9A6D75C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30912" windowHeight="15588" tabRatio="685" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1368" yWindow="1200" windowWidth="24588" windowHeight="12168" tabRatio="685" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Well settings" sheetId="1" r:id="rId1"/>
@@ -62,7 +62,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="913" uniqueCount="393">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="393">
   <si>
     <t>Select Yes or No</t>
   </si>
@@ -2091,13 +2091,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" customWidth="1"/>
+    <col min="1" max="1" width="5.6640625" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -2108,7 +2108,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -2137,7 +2137,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>21</v>
       </c>
@@ -2157,7 +2157,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -2185,7 +2185,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>21</v>
       </c>
@@ -2199,7 +2199,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -2213,7 +2213,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2233,7 +2233,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>21</v>
       </c>
@@ -2250,7 +2250,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B10" s="13"/>
       <c r="C10" s="20" t="s">
         <v>23</v>
@@ -2259,7 +2259,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C11" s="21" t="s">
         <v>35</v>
       </c>
@@ -2267,7 +2267,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C12" s="22" t="s">
         <v>37</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C13" s="23" t="s">
         <v>39</v>
       </c>
@@ -2299,18 +2299,18 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:G33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="17.42578125" customWidth="1"/>
+    <col min="1" max="1" width="17.44140625" customWidth="1"/>
     <col min="6" max="6" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F1" s="7" t="s">
         <v>300</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="33" t="s">
         <v>269</v>
       </c>
@@ -2333,7 +2333,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>303</v>
       </c>
@@ -2350,7 +2350,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>304</v>
       </c>
@@ -2373,7 +2373,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>307</v>
       </c>
@@ -2390,7 +2390,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>308</v>
       </c>
@@ -2407,7 +2407,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>309</v>
       </c>
@@ -2424,7 +2424,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>310</v>
       </c>
@@ -2441,7 +2441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>311</v>
       </c>
@@ -2458,7 +2458,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>312</v>
       </c>
@@ -2475,7 +2475,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>313</v>
       </c>
@@ -2492,7 +2492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>314</v>
       </c>
@@ -2509,7 +2509,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>315</v>
       </c>
@@ -2526,7 +2526,7 @@
         <v>270</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>316</v>
       </c>
@@ -2543,7 +2543,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>317</v>
       </c>
@@ -2560,7 +2560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>318</v>
       </c>
@@ -2577,7 +2577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>319</v>
       </c>
@@ -2594,7 +2594,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>320</v>
       </c>
@@ -2611,7 +2611,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>321</v>
       </c>
@@ -2628,7 +2628,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>322</v>
       </c>
@@ -2645,7 +2645,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>323</v>
       </c>
@@ -2662,7 +2662,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>324</v>
       </c>
@@ -2679,7 +2679,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>325</v>
       </c>
@@ -2696,7 +2696,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>326</v>
       </c>
@@ -2713,7 +2713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>327</v>
       </c>
@@ -2730,7 +2730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>328</v>
       </c>
@@ -2747,7 +2747,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>329</v>
       </c>
@@ -2764,7 +2764,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>330</v>
       </c>
@@ -2781,7 +2781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>331</v>
       </c>
@@ -2798,7 +2798,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>332</v>
       </c>
@@ -2815,7 +2815,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>333</v>
       </c>
@@ -2832,7 +2832,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>334</v>
       </c>
@@ -2849,7 +2849,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>335</v>
       </c>
@@ -2875,19 +2875,19 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:D4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="10.28515625" customWidth="1"/>
-    <col min="3" max="3" width="17.42578125" customWidth="1"/>
+    <col min="1" max="2" width="10.33203125" customWidth="1"/>
+    <col min="3" max="3" width="17.44140625" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
       <c r="D1" s="5" t="s">
         <v>336</v>
       </c>
     </row>
-    <row r="2" spans="1:4" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" s="8" customFormat="1" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>291</v>
       </c>
@@ -2901,7 +2901,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>28</v>
       </c>
@@ -2915,7 +2915,7 @@
         <v>297</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>28</v>
       </c>
@@ -2960,9 +2960,9 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCD9C215-DCD2-40A2-A7D5-172DC530BE0E}">
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
       <c r="D1" s="2"/>
@@ -2983,7 +2983,7 @@
       </c>
       <c r="O1" s="2"/>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>386</v>
       </c>
@@ -3036,9 +3036,9 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3CCC2506-3BD3-4476-A9AA-1673C259914E}">
   <dimension ref="A1:M2"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>391</v>
@@ -3051,7 +3051,7 @@
       <c r="I1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>387</v>
       </c>
@@ -3097,19 +3097,19 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
   <dimension ref="A1:Q18"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="16.28515625" customWidth="1"/>
-    <col min="3" max="3" width="12.28515625" customWidth="1"/>
-    <col min="4" max="4" width="9.85546875" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="4" max="4" width="9.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="H1" s="2" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" s="6" customFormat="1" ht="42.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="6" t="s">
         <v>338</v>
       </c>
@@ -3159,7 +3159,7 @@
         <v>362</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -3213,7 +3213,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -3264,7 +3264,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="E5" t="s">
         <v>352</v>
       </c>
@@ -3291,7 +3291,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F6" t="s">
         <v>27</v>
       </c>
@@ -3312,7 +3312,7 @@
         <v>370</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F7" t="s">
         <v>30</v>
       </c>
@@ -3330,7 +3330,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F8" t="s">
         <v>33</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F9" t="s">
         <v>24</v>
       </c>
@@ -3354,7 +3354,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F10" t="s">
         <v>36</v>
       </c>
@@ -3366,7 +3366,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F11" t="s">
         <v>38</v>
       </c>
@@ -3378,7 +3378,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F12" t="s">
         <v>40</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F13" t="s">
         <v>355</v>
       </c>
@@ -3402,7 +3402,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F14" t="s">
         <v>356</v>
       </c>
@@ -3414,7 +3414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F15" t="s">
         <v>133</v>
       </c>
@@ -3426,7 +3426,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="F16" t="s">
         <v>357</v>
       </c>
@@ -3438,7 +3438,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H17" s="30" t="s">
         <v>185</v>
       </c>
@@ -3447,7 +3447,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="8:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="8:9" x14ac:dyDescent="0.3">
       <c r="H18" s="30" t="s">
         <v>186</v>
       </c>
@@ -3465,19 +3465,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:R11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="2" width="9.7109375" style="13" customWidth="1"/>
-    <col min="3" max="3" width="15.85546875" customWidth="1"/>
-    <col min="4" max="5" width="11.5703125" customWidth="1"/>
+    <col min="1" max="2" width="9.6640625" style="13" customWidth="1"/>
+    <col min="3" max="3" width="15.88671875" customWidth="1"/>
+    <col min="4" max="5" width="11.5546875" customWidth="1"/>
     <col min="6" max="7" width="10" customWidth="1"/>
-    <col min="11" max="11" width="16.140625" customWidth="1"/>
+    <col min="11" max="11" width="16.109375" customWidth="1"/>
     <col min="13" max="13" width="7" customWidth="1"/>
-    <col min="16" max="16" width="6.5703125" customWidth="1"/>
-    <col min="17" max="17" width="4.7109375" customWidth="1"/>
+    <col min="16" max="16" width="6.5546875" customWidth="1"/>
+    <col min="17" max="17" width="4.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>41</v>
       </c>
@@ -3485,7 +3485,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:18" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
         <v>3</v>
       </c>
@@ -3541,7 +3541,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>12</v>
       </c>
@@ -3570,7 +3570,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="13" t="s">
         <v>12</v>
       </c>
@@ -3587,7 +3587,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
         <v>15</v>
       </c>
@@ -3613,7 +3613,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="13" t="s">
         <v>18</v>
       </c>
@@ -3639,7 +3639,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>22</v>
       </c>
@@ -3668,7 +3668,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="13" t="s">
         <v>25</v>
       </c>
@@ -3685,7 +3685,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
         <v>25</v>
       </c>
@@ -3708,7 +3708,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="13" t="s">
         <v>28</v>
       </c>
@@ -3740,7 +3740,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="13" t="s">
         <v>31</v>
       </c>
@@ -3794,18 +3794,18 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="5.42578125" customWidth="1"/>
+    <col min="2" max="2" width="5.44140625" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="5" width="14.85546875" customWidth="1"/>
-    <col min="6" max="6" width="13.28515625" customWidth="1"/>
+    <col min="5" max="5" width="14.88671875" customWidth="1"/>
+    <col min="6" max="6" width="13.33203125" customWidth="1"/>
     <col min="8" max="8" width="12" customWidth="1"/>
-    <col min="9" max="9" width="11.5703125" customWidth="1"/>
-    <col min="10" max="10" width="17.85546875" customWidth="1"/>
+    <col min="9" max="9" width="11.5546875" customWidth="1"/>
+    <col min="10" max="10" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>98</v>
       </c>
@@ -3821,7 +3821,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -3853,7 +3853,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>12</v>
       </c>
@@ -3885,10 +3885,10 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="13"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
         <v>15</v>
       </c>
@@ -3920,10 +3920,10 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="13"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>18</v>
       </c>
@@ -3955,10 +3955,10 @@
         <v>7</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="13"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
         <v>28</v>
       </c>
@@ -4044,19 +4044,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:O30"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.42578125" customWidth="1"/>
-    <col min="2" max="2" width="14.140625" customWidth="1"/>
-    <col min="3" max="3" width="14.5703125" customWidth="1"/>
+    <col min="1" max="1" width="11.44140625" customWidth="1"/>
+    <col min="2" max="2" width="14.109375" customWidth="1"/>
+    <col min="3" max="3" width="14.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:15" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>188</v>
       </c>
@@ -4103,7 +4103,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>202</v>
       </c>
@@ -4138,7 +4138,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>45</v>
       </c>
@@ -4170,7 +4170,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>47</v>
       </c>
@@ -4202,7 +4202,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>210</v>
       </c>
@@ -4237,7 +4237,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>213</v>
       </c>
@@ -4272,7 +4272,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>215</v>
       </c>
@@ -4307,7 +4307,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>219</v>
       </c>
@@ -4332,7 +4332,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>221</v>
       </c>
@@ -4357,7 +4357,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>222</v>
       </c>
@@ -4392,7 +4392,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>223</v>
       </c>
@@ -4427,7 +4427,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>226</v>
       </c>
@@ -4462,7 +4462,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>77</v>
       </c>
@@ -4497,7 +4497,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>228</v>
       </c>
@@ -4532,7 +4532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>231</v>
       </c>
@@ -4567,7 +4567,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>234</v>
       </c>
@@ -4602,7 +4602,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>237</v>
       </c>
@@ -4637,7 +4637,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>239</v>
       </c>
@@ -4672,7 +4672,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>241</v>
       </c>
@@ -4707,7 +4707,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>243</v>
       </c>
@@ -4745,7 +4745,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>248</v>
       </c>
@@ -4774,7 +4774,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>250</v>
       </c>
@@ -4809,7 +4809,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>254</v>
       </c>
@@ -4840,7 +4840,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>257</v>
       </c>
@@ -4875,7 +4875,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>57</v>
       </c>
@@ -4895,7 +4895,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>259</v>
       </c>
@@ -4921,7 +4921,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>260</v>
       </c>
@@ -4950,7 +4950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>262</v>
       </c>
@@ -4979,7 +4979,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>264</v>
       </c>
@@ -5019,15 +5019,15 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="6" customWidth="1"/>
-    <col min="3" max="3" width="29.28515625" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" customWidth="1"/>
-    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="3" max="3" width="29.33203125" customWidth="1"/>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
+    <col min="5" max="5" width="11.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>98</v>
       </c>
@@ -5042,7 +5042,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -5077,7 +5077,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" s="13" t="s">
         <v>12</v>
       </c>
@@ -5106,7 +5106,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" s="13" t="s">
         <v>15</v>
       </c>
@@ -5135,7 +5135,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" s="13" t="s">
         <v>18</v>
       </c>
@@ -5164,7 +5164,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" s="13" t="s">
         <v>28</v>
       </c>
@@ -5244,13 +5244,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:M17"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
-    <col min="6" max="6" width="15.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="2"/>
       <c r="B1" s="2" t="s">
         <v>124</v>
@@ -5267,7 +5267,7 @@
       <c r="I1" s="2"/>
       <c r="K1" s="2"/>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>127</v>
       </c>
@@ -5308,7 +5308,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>137</v>
       </c>
@@ -5334,7 +5334,7 @@
         <v>-18877.708702820371</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>143</v>
       </c>
@@ -5360,7 +5360,7 @@
         <v>-19045.139985898601</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>145</v>
       </c>
@@ -5386,7 +5386,7 @@
         <v>-5.4445188599886638</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>147</v>
       </c>
@@ -5412,7 +5412,7 @@
         <v>2.671411511624413</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>149</v>
       </c>
@@ -5438,7 +5438,7 @@
         <v>9.5532474786010475</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>137</v>
       </c>
@@ -5464,7 +5464,7 @@
         <v>2866.0938229725748</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>143</v>
       </c>
@@ -5490,7 +5490,7 @@
         <v>1490.761502865475</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>145</v>
       </c>
@@ -5516,7 +5516,7 @@
         <v>2.217459469264154</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>147</v>
       </c>
@@ -5542,7 +5542,7 @@
         <v>0.2337935274525294</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>149</v>
       </c>
@@ -5568,7 +5568,7 @@
         <v>2.0873115011979051E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>137</v>
       </c>
@@ -5594,7 +5594,7 @@
         <v>1351.711647219304</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>143</v>
       </c>
@@ -5620,7 +5620,7 @@
         <v>150.9391394665019</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>145</v>
       </c>
@@ -5646,7 +5646,7 @@
         <v>1.940117188288828</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>147</v>
       </c>
@@ -5672,7 +5672,7 @@
         <v>-2.0146865510893688E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>149</v>
       </c>
@@ -5706,22 +5706,22 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G42"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="16.7109375" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>165</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="5" spans="1:7" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" s="1" customFormat="1" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>2</v>
       </c>
@@ -5744,7 +5744,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>12</v>
       </c>
@@ -5764,7 +5764,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>12</v>
       </c>
@@ -5781,7 +5781,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
         <v>12</v>
       </c>
@@ -5798,7 +5798,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
         <v>12</v>
       </c>
@@ -5815,7 +5815,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
         <v>12</v>
       </c>
@@ -5832,7 +5832,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
         <v>12</v>
       </c>
@@ -5849,7 +5849,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
         <v>12</v>
       </c>
@@ -5866,7 +5866,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
         <v>15</v>
       </c>
@@ -5883,7 +5883,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
         <v>15</v>
       </c>
@@ -5900,7 +5900,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
         <v>15</v>
       </c>
@@ -5917,7 +5917,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
         <v>15</v>
       </c>
@@ -5934,7 +5934,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
         <v>15</v>
       </c>
@@ -5951,7 +5951,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="18" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
         <v>15</v>
       </c>
@@ -5968,7 +5968,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="19" spans="2:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6" hidden="1" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
         <v>15</v>
       </c>
@@ -5985,7 +5985,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
         <v>18</v>
       </c>
@@ -6002,7 +6002,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
         <v>18</v>
       </c>
@@ -6019,7 +6019,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
         <v>18</v>
       </c>
@@ -6036,7 +6036,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
         <v>18</v>
       </c>
@@ -6053,7 +6053,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
         <v>18</v>
       </c>
@@ -6070,7 +6070,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B25" t="s">
         <v>18</v>
       </c>
@@ -6087,7 +6087,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B26" t="s">
         <v>18</v>
       </c>
@@ -6104,7 +6104,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
         <v>28</v>
       </c>
@@ -6121,7 +6121,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B28" t="s">
         <v>28</v>
       </c>
@@ -6138,7 +6138,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B29" t="s">
         <v>28</v>
       </c>
@@ -6155,7 +6155,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B30" t="s">
         <v>28</v>
       </c>
@@ -6172,7 +6172,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="31" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="31" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B31" t="s">
         <v>28</v>
       </c>
@@ -6189,7 +6189,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="32" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B32" t="s">
         <v>28</v>
       </c>
@@ -6206,7 +6206,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="33" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="33" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B33" t="s">
         <v>28</v>
       </c>
@@ -6223,7 +6223,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="34" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="34" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B34" t="s">
         <v>31</v>
       </c>
@@ -6240,7 +6240,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="35" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
         <v>31</v>
       </c>
@@ -6257,7 +6257,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="36" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="36" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B36" t="s">
         <v>31</v>
       </c>
@@ -6274,7 +6274,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="37" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="37" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B37" t="s">
         <v>31</v>
       </c>
@@ -6291,7 +6291,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="38" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="38" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
         <v>31</v>
       </c>
@@ -6308,7 +6308,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="39" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="39" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B39" t="s">
         <v>31</v>
       </c>
@@ -6325,7 +6325,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="40" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="40" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B40" t="s">
         <v>31</v>
       </c>
@@ -6342,7 +6342,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="41" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="41" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B41" t="s">
         <v>31</v>
       </c>
@@ -6359,7 +6359,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="42" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="42" spans="2:6" x14ac:dyDescent="0.3">
       <c r="B42" t="s">
         <v>31</v>
       </c>
@@ -6393,25 +6393,25 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:O8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.5703125" customWidth="1"/>
+    <col min="1" max="1" width="8.5546875" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="12.85546875" customWidth="1"/>
+    <col min="3" max="3" width="12.88671875" customWidth="1"/>
     <col min="4" max="4" width="10" customWidth="1"/>
-    <col min="6" max="6" width="6.7109375" customWidth="1"/>
-    <col min="7" max="7" width="6.5703125" customWidth="1"/>
-    <col min="8" max="8" width="8.28515625" customWidth="1"/>
-    <col min="9" max="9" width="5.5703125" customWidth="1"/>
-    <col min="10" max="10" width="6.5703125" customWidth="1"/>
-    <col min="11" max="11" width="6.140625" customWidth="1"/>
-    <col min="12" max="12" width="5.140625" customWidth="1"/>
-    <col min="13" max="13" width="5.5703125" customWidth="1"/>
-    <col min="14" max="14" width="5.140625" customWidth="1"/>
-    <col min="15" max="15" width="4.42578125" customWidth="1"/>
+    <col min="6" max="6" width="6.6640625" customWidth="1"/>
+    <col min="7" max="7" width="6.5546875" customWidth="1"/>
+    <col min="8" max="8" width="8.33203125" customWidth="1"/>
+    <col min="9" max="9" width="5.5546875" customWidth="1"/>
+    <col min="10" max="10" width="6.5546875" customWidth="1"/>
+    <col min="11" max="11" width="6.109375" customWidth="1"/>
+    <col min="12" max="12" width="5.109375" customWidth="1"/>
+    <col min="13" max="13" width="5.5546875" customWidth="1"/>
+    <col min="14" max="14" width="5.109375" customWidth="1"/>
+    <col min="15" max="15" width="4.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>267</v>
       </c>
@@ -6419,7 +6419,7 @@
         <v>268</v>
       </c>
     </row>
-    <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:15" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="8" t="s">
         <v>269</v>
       </c>
@@ -6466,7 +6466,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>284</v>
       </c>
@@ -6506,7 +6506,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>287</v>
       </c>
@@ -6521,19 +6521,19 @@
         <v>288</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.3">
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
     </row>
@@ -6552,13 +6552,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="4" width="10.28515625" customWidth="1"/>
-    <col min="5" max="6" width="8.5703125" customWidth="1"/>
+    <col min="2" max="4" width="10.33203125" customWidth="1"/>
+    <col min="5" max="6" width="8.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -6566,7 +6566,7 @@
         <v>289</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" s="8" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -6592,7 +6592,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="31" t="s">
         <v>21</v>
       </c>
@@ -6607,7 +6607,7 @@
       </c>
       <c r="G3" s="32"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>21</v>
       </c>
@@ -6633,7 +6633,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>21</v>
       </c>
@@ -6659,7 +6659,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6" s="31" t="s">
         <v>21</v>
       </c>
@@ -6683,7 +6683,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -6709,7 +6709,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -6735,7 +6735,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9" s="31" t="s">
         <v>11</v>
       </c>
@@ -6759,7 +6759,83 @@
         <v>360</v>
       </c>
     </row>
-    <row r="21" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" t="s">
+        <v>295</v>
+      </c>
+      <c r="C10" t="s">
+        <v>28</v>
+      </c>
+      <c r="D10" t="s">
+        <v>173</v>
+      </c>
+      <c r="E10" t="s">
+        <v>284</v>
+      </c>
+      <c r="F10" t="s">
+        <v>352</v>
+      </c>
+      <c r="G10" t="s">
+        <v>297</v>
+      </c>
+      <c r="H10" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" t="s">
+        <v>295</v>
+      </c>
+      <c r="C11" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" t="s">
+        <v>173</v>
+      </c>
+      <c r="E11" t="s">
+        <v>284</v>
+      </c>
+      <c r="F11" t="s">
+        <v>287</v>
+      </c>
+      <c r="G11">
+        <v>0.2</v>
+      </c>
+      <c r="H11" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="31" t="s">
+        <v>11</v>
+      </c>
+      <c r="B12" s="31" t="s">
+        <v>298</v>
+      </c>
+      <c r="C12" s="31" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="31" t="s">
+        <v>173</v>
+      </c>
+      <c r="E12" s="31" t="s">
+        <v>287</v>
+      </c>
+      <c r="F12" s="31"/>
+      <c r="G12" s="31">
+        <v>1</v>
+      </c>
+      <c r="H12" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="21" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H21" t="s">
         <v>299</v>
       </c>

</xml_diff>